<commit_message>
Metodos http, req.params, req.queries, middlewares, libreria dayjs para fechas
</commit_message>
<xml_diff>
--- a/modules/06-NodeJS/libraries.xlsx
+++ b/modules/06-NodeJS/libraries.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\dev\UNIR-Full-Stack-Developer\modules\06-NodeJS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85EC13F6-594B-4781-8F36-84F728ECADFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F81B537-88C3-401C-8330-85E8FC2D10D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20430" yWindow="1035" windowWidth="18660" windowHeight="13170" xr2:uid="{6650FFD9-5CA3-4BEE-BEB2-AC127F71FC9F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6650FFD9-5CA3-4BEE-BEB2-AC127F71FC9F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>dotenv</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>manejo de ficheros</t>
+  </si>
+  <si>
+    <t>dayJS</t>
+  </si>
+  <si>
+    <t>trabajar con fechas. Ampliable por plugins</t>
   </si>
 </sst>
 </file>
@@ -110,10 +116,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -151,8 +158,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}" name="Tabla1" displayName="Tabla1" ref="A1:B4" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:B4" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}" name="Tabla1" displayName="Tabla1" ref="A1:B5" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:B5" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{37530F08-9DC3-4946-B368-38613B61BE9A}" name="LIBRERÍA"/>
     <tableColumn id="2" xr3:uid="{D6FE9D59-A186-4016-9BB1-94F80C3B109D}" name="DESC"/>
@@ -458,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21EC4682-5D5E-4CB8-B3F3-B4ACF251B76D}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
@@ -497,6 +504,14 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
log de fichero (lib node:fs). Conexión a bbdd MySQL (lib mysql2). Ejecucion de queries y devolucion de resultados. Update gitignore .env
</commit_message>
<xml_diff>
--- a/modules/06-NodeJS/libraries.xlsx
+++ b/modules/06-NodeJS/libraries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\dev\UNIR-Full-Stack-Developer\modules\06-NodeJS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F81B537-88C3-401C-8330-85E8FC2D10D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9CB9151-71D8-4F96-995B-B743FAB7287B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6650FFD9-5CA3-4BEE-BEB2-AC127F71FC9F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>dotenv</t>
   </si>
@@ -64,13 +64,19 @@
   </si>
   <si>
     <t>trabajar con fechas. Ampliable por plugins</t>
+  </si>
+  <si>
+    <t>mysql2</t>
+  </si>
+  <si>
+    <t>trabajar con BBDD mysql</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -80,15 +86,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -116,11 +113,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -158,8 +153,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}" name="Tabla1" displayName="Tabla1" ref="A1:B5" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:B5" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}" name="Tabla1" displayName="Tabla1" ref="A1:B6" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:B6" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{37530F08-9DC3-4946-B368-38613B61BE9A}" name="LIBRERÍA"/>
     <tableColumn id="2" xr3:uid="{D6FE9D59-A186-4016-9BB1-94F80C3B109D}" name="DESC"/>
@@ -465,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21EC4682-5D5E-4CB8-B3F3-B4ACF251B76D}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
@@ -473,7 +468,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -505,11 +500,19 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
registro de usuarios, login, tokens
</commit_message>
<xml_diff>
--- a/modules/06-NodeJS/libraries.xlsx
+++ b/modules/06-NodeJS/libraries.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\dev\UNIR-Full-Stack-Developer\modules\06-NodeJS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9CB9151-71D8-4F96-995B-B743FAB7287B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A8D957-FB9D-4AFA-AA7C-79B06E81DC07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6650FFD9-5CA3-4BEE-BEB2-AC127F71FC9F}"/>
+    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{6650FFD9-5CA3-4BEE-BEB2-AC127F71FC9F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>dotenv</t>
   </si>
@@ -70,6 +70,18 @@
   </si>
   <si>
     <t>trabajar con BBDD mysql</t>
+  </si>
+  <si>
+    <t>bcryptjs</t>
+  </si>
+  <si>
+    <t>Encriptar contraseñas</t>
+  </si>
+  <si>
+    <t>jsonwebtoken</t>
+  </si>
+  <si>
+    <t>generar web tokens</t>
   </si>
 </sst>
 </file>
@@ -113,9 +125,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -153,8 +166,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}" name="Tabla1" displayName="Tabla1" ref="A1:B6" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:B6" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}" name="Tabla1" displayName="Tabla1" ref="A1:B8" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:B8" xr:uid="{8C0FB0C7-4B0E-4565-96A1-146D8E40CB16}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{37530F08-9DC3-4946-B368-38613B61BE9A}" name="LIBRERÍA"/>
     <tableColumn id="2" xr3:uid="{D6FE9D59-A186-4016-9BB1-94F80C3B109D}" name="DESC"/>
@@ -460,10 +473,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21EC4682-5D5E-4CB8-B3F3-B4ACF251B76D}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -514,6 +527,25 @@
       <c r="B6" t="s">
         <v>11</v>
       </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>